<commit_message>
fix details prospeccion y mapas
</commit_message>
<xml_diff>
--- a/reporte_Prospeccion.xlsx
+++ b/reporte_Prospeccion.xlsx
@@ -570,15 +570,15 @@
     <col width="37" customWidth="1" style="12" min="13" max="13"/>
     <col width="43" customWidth="1" style="12" min="14" max="14"/>
     <col width="29" customWidth="1" style="12" min="15" max="15"/>
-    <col width="20" customWidth="1" style="12" min="16" max="16"/>
-    <col width="13" customWidth="1" style="12" min="17" max="18"/>
+    <col width="20" customWidth="1" style="12" min="16" max="17"/>
+    <col width="20.57" customWidth="1" style="12" min="18" max="18"/>
     <col width="30" customWidth="1" style="12" min="19" max="19"/>
     <col width="35" customWidth="1" style="12" min="20" max="20"/>
     <col width="42" customWidth="1" style="12" min="21" max="21"/>
-    <col width="27" customWidth="1" style="12" min="22" max="22"/>
+    <col width="32.57" customWidth="1" style="12" min="22" max="22"/>
     <col width="28" customWidth="1" style="12" min="23" max="23"/>
     <col width="42" customWidth="1" style="12" min="24" max="24"/>
-    <col width="27" customWidth="1" style="12" min="25" max="25"/>
+    <col width="31.43" customWidth="1" style="12" min="25" max="25"/>
     <col width="25" customWidth="1" style="12" min="26" max="26"/>
     <col width="55" customWidth="1" style="12" min="27" max="27"/>
   </cols>
@@ -589,7 +589,7 @@
         <is>
           <t>Empresa: BBVA
 Usuario: Uriel Meneses
-Fecha de descarga: 12-03-2026
+Fecha de descarga: 13-03-2026
 Descarga por Fecha de publicación del 2026-01-01 al 2026-01-31</t>
         </is>
       </c>

</xml_diff>